<commit_message>
Day 1 of Excel
</commit_message>
<xml_diff>
--- a/Day 1 Excel.xlsx
+++ b/Day 1 Excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Naik Balkrushna Anil\OneDrive\Attachments\Desktop\Exploring Data Science Field\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AA1AA56-BBFD-40F4-A7D8-9A98D0152B2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D619B89C-A52C-48A7-8C40-185303433643}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{AF654A27-534B-4126-81F4-87182200E9A0}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="16">
   <si>
     <t>Day 1 of Learning Basics of Excel</t>
   </si>
@@ -71,13 +71,16 @@
   </si>
   <si>
     <t>Average</t>
+  </si>
+  <si>
+    <t>Alignment, colors and font in Excel</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -109,6 +112,47 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Roboto"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="11"/>
+      <color theme="5" tint="-0.249977111117893"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="11"/>
+      <color theme="4"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF00B050"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF00B050"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -253,26 +297,77 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -596,210 +691,411 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB435CEE-69D2-4383-9821-50CE7ECA064E}">
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:J25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.88671875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
+      <c r="H1" s="10"/>
+      <c r="I1" s="10"/>
+      <c r="J1" s="10"/>
     </row>
     <row r="2" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="E3" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="12" t="s">
+      <c r="F3" s="16" t="s">
         <v>13</v>
       </c>
+      <c r="G3" s="17"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="6">
+      <c r="B4">
         <v>99</v>
       </c>
-      <c r="C4" s="6">
+      <c r="C4">
         <v>90</v>
       </c>
-      <c r="D4" s="6">
+      <c r="D4">
         <v>91</v>
       </c>
-      <c r="E4" s="6">
+      <c r="E4">
         <v>94</v>
       </c>
-      <c r="F4" s="9">
+      <c r="F4" s="4">
         <v>89</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A5" s="13" t="s">
+      <c r="A5" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="6">
+      <c r="B5">
         <v>81</v>
       </c>
-      <c r="C5" s="6">
+      <c r="C5">
         <v>34</v>
       </c>
-      <c r="D5" s="6">
+      <c r="D5">
         <v>76</v>
       </c>
-      <c r="E5" s="6">
+      <c r="E5">
         <v>87</v>
       </c>
-      <c r="F5" s="9">
+      <c r="F5" s="4">
         <v>98</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A6" s="13" t="s">
+      <c r="A6" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="6">
+      <c r="B6">
         <v>76</v>
       </c>
-      <c r="C6" s="6">
+      <c r="C6">
         <v>65</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D6">
         <v>75</v>
       </c>
-      <c r="E6" s="6">
+      <c r="E6">
         <v>67</v>
       </c>
-      <c r="F6" s="9">
+      <c r="F6" s="4">
         <v>87</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A7" s="13" t="s">
+      <c r="A7" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="6">
+      <c r="B7">
         <v>45</v>
       </c>
-      <c r="C7" s="6">
+      <c r="C7">
         <v>76</v>
       </c>
-      <c r="D7" s="6">
+      <c r="D7">
         <v>64</v>
       </c>
-      <c r="E7" s="6">
+      <c r="E7">
         <v>56</v>
       </c>
-      <c r="F7" s="9">
+      <c r="F7" s="4">
         <v>78</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A8" s="13" t="s">
+      <c r="A8" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="6">
+      <c r="B8">
         <v>89</v>
       </c>
-      <c r="C8" s="6">
+      <c r="C8">
         <v>83</v>
       </c>
-      <c r="D8" s="6">
+      <c r="D8">
         <v>67</v>
       </c>
-      <c r="E8" s="6">
+      <c r="E8">
         <v>45</v>
       </c>
-      <c r="F8" s="9">
+      <c r="F8" s="4">
         <v>78</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A9" s="13" t="s">
+      <c r="A9" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="6">
+      <c r="B9">
         <v>67</v>
       </c>
-      <c r="C9" s="6">
+      <c r="C9">
         <v>34</v>
       </c>
-      <c r="D9" s="6">
+      <c r="D9">
         <v>56</v>
       </c>
-      <c r="E9" s="6">
+      <c r="E9">
         <v>56</v>
       </c>
-      <c r="F9" s="9">
+      <c r="F9" s="4">
         <v>98</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="14" t="s">
+      <c r="A10" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="10">
+      <c r="B10" s="5">
         <v>83</v>
       </c>
-      <c r="C10" s="10">
+      <c r="C10" s="5">
         <v>86</v>
       </c>
-      <c r="D10" s="10">
+      <c r="D10" s="5">
         <v>87</v>
       </c>
-      <c r="E10" s="10">
+      <c r="E10" s="5">
         <v>98</v>
       </c>
-      <c r="F10" s="11">
+      <c r="F10" s="6">
         <v>67</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="4" t="s">
+      <c r="A12" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B12" s="3">
+      <c r="B12" s="1">
         <v>77.142857140000004</v>
       </c>
-      <c r="C12" s="3">
+      <c r="C12" s="1">
         <v>66.857142859999996</v>
       </c>
-      <c r="D12" s="3">
+      <c r="D12" s="1">
         <v>73.714285709999999</v>
       </c>
-      <c r="E12" s="3">
+      <c r="E12" s="1">
         <v>71.857142859999996</v>
       </c>
-      <c r="F12" s="5">
+      <c r="F12" s="3">
         <v>85</v>
       </c>
     </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A14" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="B14" s="13"/>
+      <c r="C14" s="13"/>
+      <c r="D14" s="13"/>
+      <c r="E14" s="13"/>
+      <c r="F14" s="13"/>
+    </row>
+    <row r="15" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="13"/>
+      <c r="B15" s="13"/>
+      <c r="C15" s="13"/>
+      <c r="D15" s="13"/>
+      <c r="E15" s="13"/>
+      <c r="F15" s="13"/>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A16" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="B16" s="22" t="s">
+        <v>2</v>
+      </c>
+      <c r="C16" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="D16" s="22" t="s">
+        <v>4</v>
+      </c>
+      <c r="E16" s="22" t="s">
+        <v>5</v>
+      </c>
+      <c r="F16" s="23" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A17" s="24" t="s">
+        <v>6</v>
+      </c>
+      <c r="B17" s="11">
+        <v>99</v>
+      </c>
+      <c r="C17" s="11">
+        <v>90</v>
+      </c>
+      <c r="D17" s="11">
+        <v>91</v>
+      </c>
+      <c r="E17" s="11">
+        <v>94</v>
+      </c>
+      <c r="F17" s="18">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A18" s="24" t="s">
+        <v>7</v>
+      </c>
+      <c r="B18" s="11">
+        <v>81</v>
+      </c>
+      <c r="C18" s="11">
+        <v>34</v>
+      </c>
+      <c r="D18" s="11">
+        <v>76</v>
+      </c>
+      <c r="E18" s="11">
+        <v>87</v>
+      </c>
+      <c r="F18" s="18">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A19" s="24" t="s">
+        <v>8</v>
+      </c>
+      <c r="B19" s="11">
+        <v>76</v>
+      </c>
+      <c r="C19" s="11">
+        <v>65</v>
+      </c>
+      <c r="D19" s="11">
+        <v>75</v>
+      </c>
+      <c r="E19" s="11">
+        <v>67</v>
+      </c>
+      <c r="F19" s="18">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A20" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="B20" s="11">
+        <v>45</v>
+      </c>
+      <c r="C20" s="11">
+        <v>76</v>
+      </c>
+      <c r="D20" s="11">
+        <v>64</v>
+      </c>
+      <c r="E20" s="11">
+        <v>56</v>
+      </c>
+      <c r="F20" s="18">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A21" s="24" t="s">
+        <v>10</v>
+      </c>
+      <c r="B21" s="11">
+        <v>89</v>
+      </c>
+      <c r="C21" s="11">
+        <v>83</v>
+      </c>
+      <c r="D21" s="11">
+        <v>67</v>
+      </c>
+      <c r="E21" s="11">
+        <v>45</v>
+      </c>
+      <c r="F21" s="18">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A22" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="B22" s="11">
+        <v>67</v>
+      </c>
+      <c r="C22" s="11">
+        <v>34</v>
+      </c>
+      <c r="D22" s="11">
+        <v>56</v>
+      </c>
+      <c r="E22" s="11">
+        <v>56</v>
+      </c>
+      <c r="F22" s="18">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="25" t="s">
+        <v>12</v>
+      </c>
+      <c r="B23" s="19">
+        <v>83</v>
+      </c>
+      <c r="C23" s="19">
+        <v>86</v>
+      </c>
+      <c r="D23" s="19">
+        <v>87</v>
+      </c>
+      <c r="E23" s="19">
+        <v>98</v>
+      </c>
+      <c r="F23" s="20">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A25" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="B25" s="27">
+        <v>77.142857140000004</v>
+      </c>
+      <c r="C25" s="27">
+        <v>66.857142859999996</v>
+      </c>
+      <c r="D25" s="27">
+        <v>73.714285709999999</v>
+      </c>
+      <c r="E25" s="27">
+        <v>71.857142859999996</v>
+      </c>
+      <c r="F25" s="28">
+        <v>85</v>
+      </c>
+      <c r="G25" s="29"/>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A14:F15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Day 1 of Learning Basic of Excel
</commit_message>
<xml_diff>
--- a/Day 1 Excel.xlsx
+++ b/Day 1 Excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Naik Balkrushna Anil\OneDrive\Attachments\Desktop\Exploring Data Science Field\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D619B89C-A52C-48A7-8C40-185303433643}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FB728EC-C8AA-4643-8B41-AA7464AEB340}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{AF654A27-534B-4126-81F4-87182200E9A0}"/>
   </bookViews>
@@ -80,7 +80,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -120,10 +120,15 @@
       <name val="Roboto"/>
     </font>
     <font>
-      <b/>
-      <u/>
       <sz val="11"/>
-      <color theme="5" tint="-0.249977111117893"/>
+      <color rgb="FF00B050"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -132,34 +137,36 @@
       <b/>
       <u/>
       <sz val="11"/>
-      <color theme="4"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF00B050"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF00B050"/>
+      <color theme="0"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1" tint="0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="12">
@@ -297,7 +304,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
@@ -307,67 +314,70 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -695,43 +705,44 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="19.88671875" customWidth="1"/>
+    <col min="2" max="4" width="8.88671875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
-      <c r="H1" s="10"/>
-      <c r="I1" s="10"/>
-      <c r="J1" s="10"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
+      <c r="I1" s="15"/>
+      <c r="J1" s="15"/>
     </row>
     <row r="2" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A3" s="14" t="s">
+      <c r="A3" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="15" t="s">
+      <c r="B3" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="15" t="s">
+      <c r="C3" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="D3" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="15" t="s">
+      <c r="E3" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="16" t="s">
+      <c r="F3" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="G3" s="17"/>
+      <c r="G3" s="12"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
@@ -894,203 +905,203 @@
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="12" t="s">
+      <c r="A14" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="B14" s="13"/>
-      <c r="C14" s="13"/>
-      <c r="D14" s="13"/>
-      <c r="E14" s="13"/>
-      <c r="F14" s="13"/>
+      <c r="B14" s="17"/>
+      <c r="C14" s="17"/>
+      <c r="D14" s="17"/>
+      <c r="E14" s="17"/>
+      <c r="F14" s="17"/>
     </row>
     <row r="15" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="13"/>
-      <c r="B15" s="13"/>
-      <c r="C15" s="13"/>
-      <c r="D15" s="13"/>
-      <c r="E15" s="13"/>
-      <c r="F15" s="13"/>
+      <c r="A15" s="17"/>
+      <c r="B15" s="17"/>
+      <c r="C15" s="17"/>
+      <c r="D15" s="17"/>
+      <c r="E15" s="17"/>
+      <c r="F15" s="17"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="21" t="s">
+      <c r="A16" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="B16" s="22" t="s">
+      <c r="B16" s="23" t="s">
         <v>2</v>
       </c>
-      <c r="C16" s="22" t="s">
+      <c r="C16" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="D16" s="22" t="s">
+      <c r="D16" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="E16" s="22" t="s">
+      <c r="E16" s="23" t="s">
         <v>5</v>
       </c>
-      <c r="F16" s="23" t="s">
+      <c r="F16" s="24" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A17" s="24" t="s">
+      <c r="A17" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="B17" s="11">
+      <c r="B17" s="30">
         <v>99</v>
       </c>
-      <c r="C17" s="11">
+      <c r="C17" s="18">
         <v>90</v>
       </c>
-      <c r="D17" s="11">
+      <c r="D17" s="18">
         <v>91</v>
       </c>
-      <c r="E17" s="11">
+      <c r="E17" s="18">
         <v>94</v>
       </c>
-      <c r="F17" s="18">
+      <c r="F17" s="19">
         <v>89</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A18" s="24" t="s">
+      <c r="A18" s="25" t="s">
         <v>7</v>
       </c>
-      <c r="B18" s="11">
+      <c r="B18" s="18">
         <v>81</v>
       </c>
-      <c r="C18" s="11">
+      <c r="C18" s="18">
         <v>34</v>
       </c>
-      <c r="D18" s="11">
+      <c r="D18" s="18">
         <v>76</v>
       </c>
-      <c r="E18" s="11">
+      <c r="E18" s="18">
         <v>87</v>
       </c>
-      <c r="F18" s="18">
+      <c r="F18" s="30">
         <v>98</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A19" s="24" t="s">
+      <c r="A19" s="25" t="s">
         <v>8</v>
       </c>
-      <c r="B19" s="11">
+      <c r="B19" s="18">
         <v>76</v>
       </c>
-      <c r="C19" s="11">
+      <c r="C19" s="18">
         <v>65</v>
       </c>
-      <c r="D19" s="11">
+      <c r="D19" s="18">
         <v>75</v>
       </c>
-      <c r="E19" s="11">
+      <c r="E19" s="18">
         <v>67</v>
       </c>
-      <c r="F19" s="18">
+      <c r="F19" s="19">
         <v>87</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A20" s="24" t="s">
+      <c r="A20" s="25" t="s">
         <v>9</v>
       </c>
-      <c r="B20" s="11">
+      <c r="B20" s="18">
         <v>45</v>
       </c>
-      <c r="C20" s="11">
+      <c r="C20" s="18">
         <v>76</v>
       </c>
-      <c r="D20" s="11">
+      <c r="D20" s="18">
         <v>64</v>
       </c>
-      <c r="E20" s="11">
+      <c r="E20" s="18">
         <v>56</v>
       </c>
-      <c r="F20" s="18">
+      <c r="F20" s="19">
         <v>78</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A21" s="24" t="s">
+      <c r="A21" s="25" t="s">
         <v>10</v>
       </c>
-      <c r="B21" s="11">
+      <c r="B21" s="18">
         <v>89</v>
       </c>
-      <c r="C21" s="11">
+      <c r="C21" s="18">
         <v>83</v>
       </c>
-      <c r="D21" s="11">
+      <c r="D21" s="18">
         <v>67</v>
       </c>
-      <c r="E21" s="11">
+      <c r="E21" s="18">
         <v>45</v>
       </c>
-      <c r="F21" s="18">
+      <c r="F21" s="19">
         <v>78</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A22" s="24" t="s">
+      <c r="A22" s="25" t="s">
         <v>11</v>
       </c>
-      <c r="B22" s="11">
+      <c r="B22" s="18">
         <v>67</v>
       </c>
-      <c r="C22" s="11">
+      <c r="C22" s="18">
         <v>34</v>
       </c>
-      <c r="D22" s="11">
+      <c r="D22" s="18">
         <v>56</v>
       </c>
-      <c r="E22" s="11">
+      <c r="E22" s="18">
         <v>56</v>
       </c>
-      <c r="F22" s="18">
+      <c r="F22" s="30">
         <v>98</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="25" t="s">
+      <c r="A23" s="26" t="s">
         <v>12</v>
       </c>
-      <c r="B23" s="19">
+      <c r="B23" s="20">
         <v>83</v>
       </c>
-      <c r="C23" s="19">
+      <c r="C23" s="20">
         <v>86</v>
       </c>
-      <c r="D23" s="19">
+      <c r="D23" s="20">
         <v>87</v>
       </c>
-      <c r="E23" s="19">
+      <c r="E23" s="20">
         <v>98</v>
       </c>
-      <c r="F23" s="20">
+      <c r="F23" s="21">
         <v>67</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A25" s="26" t="s">
+      <c r="A25" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="B25" s="27">
+      <c r="B25" s="28">
         <v>77.142857140000004</v>
       </c>
-      <c r="C25" s="27">
+      <c r="C25" s="28">
         <v>66.857142859999996</v>
       </c>
-      <c r="D25" s="27">
+      <c r="D25" s="28">
         <v>73.714285709999999</v>
       </c>
-      <c r="E25" s="27">
+      <c r="E25" s="28">
         <v>71.857142859999996</v>
       </c>
-      <c r="F25" s="28">
+      <c r="F25" s="29">
         <v>85</v>
       </c>
-      <c r="G25" s="29"/>
+      <c r="G25" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>